<commit_message>
Update placeholder Excel file with new data
</commit_message>
<xml_diff>
--- a/homework2.xlsx
+++ b/homework2.xlsx
@@ -5,7 +5,7 @@
   <workbookPr hidePivotFieldList="1" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\disco\Documents\DataAnalytics-2026\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/634f1a5acd5bf9fd/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="175" documentId="8_{EF02D1D8-E723-4C92-8CB9-388DFEC8DDF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FE9F2FBF-3C69-4F20-ACD0-93E2772D0FE6}"/>
@@ -510,7 +510,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000001-D085-4BCF-BF15-4C7ED001C797}"/>
+                <c16:uniqueId val="{00000001-1CEB-47F5-9EFA-AFAF648F43F0}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -534,7 +534,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000003-D085-4BCF-BF15-4C7ED001C797}"/>
+                <c16:uniqueId val="{00000003-1CEB-47F5-9EFA-AFAF648F43F0}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -558,7 +558,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000005-D085-4BCF-BF15-4C7ED001C797}"/>
+                <c16:uniqueId val="{00000005-1CEB-47F5-9EFA-AFAF648F43F0}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -582,7 +582,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000007-D085-4BCF-BF15-4C7ED001C797}"/>
+                <c16:uniqueId val="{00000007-1CEB-47F5-9EFA-AFAF648F43F0}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -1039,7 +1039,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000001-D7FD-49A2-A351-97BF4F050DA0}"/>
+                <c16:uniqueId val="{00000001-49DE-4254-B1BD-D2AEA0059709}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -1063,7 +1063,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000003-D7FD-49A2-A351-97BF4F050DA0}"/>
+                <c16:uniqueId val="{00000003-49DE-4254-B1BD-D2AEA0059709}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -1087,7 +1087,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000005-D7FD-49A2-A351-97BF4F050DA0}"/>
+                <c16:uniqueId val="{00000005-49DE-4254-B1BD-D2AEA0059709}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>

</xml_diff>